<commit_message>
New V1.0 KG100 Sensor data sheet
New Data sheet for KG100 sensor with external transmitter V1.0
</commit_message>
<xml_diff>
--- a/Images for Markdown files database updated 30-06-2026.xlsx
+++ b/Images for Markdown files database updated 30-06-2026.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\trevor\Compac Industries\Compac - General\IT\ChatBot\Markdown-Manuals\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6D63C21F-BA2B-40B3-BFB0-CDDAF74F31D3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A79180CE-AC70-488B-8565-67D67F380E09}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-38520" yWindow="-1320" windowWidth="38640" windowHeight="21120" xr2:uid="{7323B22B-375C-41F7-91CD-F86C900FC6DE}"/>
   </bookViews>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1014" uniqueCount="562">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1051" uniqueCount="588">
   <si>
     <t xml:space="preserve">PCBs </t>
   </si>
@@ -1730,6 +1730,84 @@
   </si>
   <si>
     <t>17.1.1_KG100_dims.png</t>
+  </si>
+  <si>
+    <t>18.1.1</t>
+  </si>
+  <si>
+    <t>18.1.2</t>
+  </si>
+  <si>
+    <t>18.1.3</t>
+  </si>
+  <si>
+    <t>18.1.4</t>
+  </si>
+  <si>
+    <t>18.1.5</t>
+  </si>
+  <si>
+    <t>18.2.1</t>
+  </si>
+  <si>
+    <t>Sensors with built-in Transmitter</t>
+  </si>
+  <si>
+    <t>Sensor with External Transmitter</t>
+  </si>
+  <si>
+    <t>18.2.2</t>
+  </si>
+  <si>
+    <t>18.2.3</t>
+  </si>
+  <si>
+    <t>18.2.4</t>
+  </si>
+  <si>
+    <t>18.2.5</t>
+  </si>
+  <si>
+    <t>Sensor with Fluid Control System</t>
+  </si>
+  <si>
+    <t>18.3.1</t>
+  </si>
+  <si>
+    <t>18.3.2</t>
+  </si>
+  <si>
+    <t>18.3.3</t>
+  </si>
+  <si>
+    <t>18.3.4</t>
+  </si>
+  <si>
+    <t>18.3.5</t>
+  </si>
+  <si>
+    <t>Sensor and transmitter</t>
+  </si>
+  <si>
+    <t>Sensor and transmitter angle view</t>
+  </si>
+  <si>
+    <t>Sensor with external trans display</t>
+  </si>
+  <si>
+    <t>18.2.1_Sensor_and_Transmitter.png</t>
+  </si>
+  <si>
+    <t>18.2.2_Sensor_and_Transmitter_angle.png</t>
+  </si>
+  <si>
+    <t>18.2.3_Sensor_and_Transmitter_display.png</t>
+  </si>
+  <si>
+    <t>Approvals and standards emblems</t>
+  </si>
+  <si>
+    <t>18.2.4_Sensor_and_Transmitter_approvals.png</t>
   </si>
 </sst>
 </file>
@@ -2209,15 +2287,15 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2B533B56-556A-40A2-8D3F-E8E5A852019A}">
-  <dimension ref="A1:G224"/>
+  <dimension ref="A1:G242"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="11.26953125" style="1" customWidth="1"/>
-    <col min="2" max="2" width="26.7265625" customWidth="1"/>
+    <col min="2" max="2" width="30.7265625" customWidth="1"/>
     <col min="3" max="3" width="10.6328125" style="1" customWidth="1"/>
     <col min="4" max="4" width="47.26953125" customWidth="1"/>
     <col min="5" max="5" width="16" style="1" customWidth="1"/>
-    <col min="6" max="6" width="24.1796875" customWidth="1"/>
+    <col min="6" max="6" width="29.81640625" customWidth="1"/>
     <col min="7" max="7" width="13.81640625" customWidth="1"/>
   </cols>
   <sheetData>
@@ -5379,6 +5457,233 @@
       <c r="E224" s="4"/>
       <c r="F224" s="5"/>
       <c r="G224" s="5"/>
+    </row>
+    <row r="226" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A226" s="4"/>
+      <c r="B226" s="5" t="s">
+        <v>568</v>
+      </c>
+      <c r="C226" s="4" t="s">
+        <v>562</v>
+      </c>
+      <c r="D226" s="16" t="s">
+        <v>562</v>
+      </c>
+      <c r="E226" s="4"/>
+      <c r="F226" s="5"/>
+      <c r="G226" s="5"/>
+    </row>
+    <row r="227" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A227" s="4"/>
+      <c r="B227" s="5"/>
+      <c r="C227" s="4" t="s">
+        <v>563</v>
+      </c>
+      <c r="D227" s="16" t="s">
+        <v>563</v>
+      </c>
+      <c r="E227" s="4"/>
+      <c r="F227" s="5"/>
+      <c r="G227" s="5"/>
+    </row>
+    <row r="228" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A228" s="4"/>
+      <c r="B228" s="5"/>
+      <c r="C228" s="4" t="s">
+        <v>564</v>
+      </c>
+      <c r="D228" s="16" t="s">
+        <v>564</v>
+      </c>
+      <c r="E228" s="4"/>
+      <c r="F228" s="5"/>
+      <c r="G228" s="5"/>
+    </row>
+    <row r="229" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A229" s="4"/>
+      <c r="B229" s="5"/>
+      <c r="C229" s="4" t="s">
+        <v>565</v>
+      </c>
+      <c r="D229" s="16" t="s">
+        <v>565</v>
+      </c>
+      <c r="E229" s="4"/>
+      <c r="F229" s="5"/>
+      <c r="G229" s="5"/>
+    </row>
+    <row r="230" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A230" s="4"/>
+      <c r="B230" s="5"/>
+      <c r="C230" s="4" t="s">
+        <v>566</v>
+      </c>
+      <c r="D230" s="16" t="s">
+        <v>566</v>
+      </c>
+      <c r="E230" s="4"/>
+      <c r="F230" s="5"/>
+      <c r="G230" s="5"/>
+    </row>
+    <row r="231" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A231" s="4"/>
+      <c r="B231" s="5"/>
+      <c r="C231" s="4"/>
+      <c r="D231" s="5"/>
+      <c r="E231" s="4"/>
+      <c r="F231" s="5"/>
+      <c r="G231" s="5"/>
+    </row>
+    <row r="232" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A232" s="4"/>
+      <c r="B232" s="5" t="s">
+        <v>569</v>
+      </c>
+      <c r="C232" s="4" t="s">
+        <v>567</v>
+      </c>
+      <c r="D232" s="16" t="s">
+        <v>583</v>
+      </c>
+      <c r="E232" s="4"/>
+      <c r="F232" s="5" t="s">
+        <v>580</v>
+      </c>
+      <c r="G232" s="5"/>
+    </row>
+    <row r="233" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A233" s="4"/>
+      <c r="B233" s="5"/>
+      <c r="C233" s="4" t="s">
+        <v>570</v>
+      </c>
+      <c r="D233" s="16" t="s">
+        <v>584</v>
+      </c>
+      <c r="E233" s="4"/>
+      <c r="F233" s="5" t="s">
+        <v>581</v>
+      </c>
+      <c r="G233" s="5"/>
+    </row>
+    <row r="234" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A234" s="4"/>
+      <c r="B234" s="5"/>
+      <c r="C234" s="4" t="s">
+        <v>571</v>
+      </c>
+      <c r="D234" s="16" t="s">
+        <v>585</v>
+      </c>
+      <c r="E234" s="4"/>
+      <c r="F234" s="5" t="s">
+        <v>582</v>
+      </c>
+      <c r="G234" s="5"/>
+    </row>
+    <row r="235" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A235" s="4"/>
+      <c r="B235" s="5"/>
+      <c r="C235" s="4" t="s">
+        <v>572</v>
+      </c>
+      <c r="D235" s="16" t="s">
+        <v>587</v>
+      </c>
+      <c r="E235" s="4"/>
+      <c r="F235" s="5" t="s">
+        <v>586</v>
+      </c>
+      <c r="G235" s="5"/>
+    </row>
+    <row r="236" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A236" s="4"/>
+      <c r="B236" s="5"/>
+      <c r="C236" s="4" t="s">
+        <v>573</v>
+      </c>
+      <c r="D236" s="16" t="s">
+        <v>573</v>
+      </c>
+      <c r="E236" s="4"/>
+      <c r="F236" s="5"/>
+      <c r="G236" s="5"/>
+    </row>
+    <row r="237" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A237" s="4"/>
+      <c r="B237" s="5"/>
+      <c r="C237" s="4"/>
+      <c r="D237" s="5"/>
+      <c r="E237" s="4"/>
+      <c r="F237" s="5"/>
+      <c r="G237" s="5"/>
+    </row>
+    <row r="238" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A238" s="4"/>
+      <c r="B238" s="5" t="s">
+        <v>574</v>
+      </c>
+      <c r="C238" s="4" t="s">
+        <v>575</v>
+      </c>
+      <c r="D238" s="16" t="s">
+        <v>575</v>
+      </c>
+      <c r="E238" s="4"/>
+      <c r="F238" s="5"/>
+      <c r="G238" s="5"/>
+    </row>
+    <row r="239" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A239" s="4"/>
+      <c r="B239" s="5"/>
+      <c r="C239" s="4" t="s">
+        <v>576</v>
+      </c>
+      <c r="D239" s="16" t="s">
+        <v>576</v>
+      </c>
+      <c r="E239" s="4"/>
+      <c r="F239" s="5"/>
+      <c r="G239" s="5"/>
+    </row>
+    <row r="240" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A240" s="4"/>
+      <c r="B240" s="5"/>
+      <c r="C240" s="4" t="s">
+        <v>577</v>
+      </c>
+      <c r="D240" s="16" t="s">
+        <v>577</v>
+      </c>
+      <c r="E240" s="4"/>
+      <c r="F240" s="5"/>
+      <c r="G240" s="5"/>
+    </row>
+    <row r="241" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A241" s="4"/>
+      <c r="B241" s="5"/>
+      <c r="C241" s="4" t="s">
+        <v>578</v>
+      </c>
+      <c r="D241" s="16" t="s">
+        <v>578</v>
+      </c>
+      <c r="E241" s="4"/>
+      <c r="F241" s="5"/>
+      <c r="G241" s="5"/>
+    </row>
+    <row r="242" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A242" s="4"/>
+      <c r="B242" s="5"/>
+      <c r="C242" s="4" t="s">
+        <v>579</v>
+      </c>
+      <c r="D242" s="16" t="s">
+        <v>579</v>
+      </c>
+      <c r="E242" s="4"/>
+      <c r="F242" s="5"/>
+      <c r="G242" s="5"/>
     </row>
   </sheetData>
   <phoneticPr fontId="2" type="noConversion"/>

</xml_diff>